<commit_message>
--27/05--Dũng-- update export excel theo mẫu v1
</commit_message>
<xml_diff>
--- a/BCEndlineNgay (22)_Empty.xlsx
+++ b/BCEndlineNgay (22)_Empty.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leuti\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leuti\Desktop\GitHub\Demo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37D5A7FA-C520-42EB-98AC-F20682AC2E0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57A1F3DF-4757-44A8-B5C4-087A32205DC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1023,14 +1023,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>201231</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>257175</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>181421</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>

</xml_diff>